<commit_message>
Actualización automática: 2026-09-30 14:53:37
</commit_message>
<xml_diff>
--- a/Inventory/dynamic_inventory/inventory_data.xlsx
+++ b/Inventory/dynamic_inventory/inventory_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\7167351\AppData\Local\Temp\scp11124\ansible\CIS-Ansible\Inventory\dynamic_inventory\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\7167351\AppData\Local\Temp\scp29226\ansible\CIS-Ansible\Inventory\dynamic_inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61ABB964-9606-4A58-9F2B-121D59ABF680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAE5C25-C514-46DB-913A-FC4F365BE3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="299">
   <si>
     <t>Host</t>
   </si>
@@ -911,6 +911,12 @@
   </si>
   <si>
     <t>plantillaol9</t>
+  </si>
+  <si>
+    <t>opshiftbastrh9</t>
+  </si>
+  <si>
+    <t>10.181.40.12</t>
   </si>
 </sst>
 </file>
@@ -1287,11 +1293,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.08203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -3622,6 +3629,23 @@
       </c>
       <c r="E136" t="s">
         <v>296</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>298</v>
+      </c>
+      <c r="B137" t="s">
+        <v>297</v>
+      </c>
+      <c r="C137" t="s">
+        <v>298</v>
+      </c>
+      <c r="D137" t="s">
+        <v>8</v>
+      </c>
+      <c r="E137" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática: 2026-10-14 10:36:03
</commit_message>
<xml_diff>
--- a/Inventory/dynamic_inventory/inventory_data.xlsx
+++ b/Inventory/dynamic_inventory/inventory_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\7167351\AppData\Local\Temp\scp29226\ansible\CIS-Ansible\Inventory\dynamic_inventory\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\79958935\AppData\Local\Temp\scp32174\ansible\CIS-Ansible\Inventory\dynamic_inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAE5C25-C514-46DB-913A-FC4F365BE3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CD3BF3-1CD7-4AAE-BB4C-906AAF2E38E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="303">
   <si>
     <t>Host</t>
   </si>
@@ -917,6 +917,18 @@
   </si>
   <si>
     <t>10.181.40.12</t>
+  </si>
+  <si>
+    <t>10.0.16.69</t>
+  </si>
+  <si>
+    <t>VM-EU2-DBMANH01-PRD</t>
+  </si>
+  <si>
+    <t>azureuser</t>
+  </si>
+  <si>
+    <t>dbmanhattan</t>
   </si>
 </sst>
 </file>
@@ -1293,12 +1305,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.08203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.1640625" customWidth="1"/>
+    <col min="5" max="5" width="22.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -3646,6 +3659,23 @@
       </c>
       <c r="E137" t="s">
         <v>297</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>299</v>
+      </c>
+      <c r="B138" t="s">
+        <v>300</v>
+      </c>
+      <c r="C138" t="s">
+        <v>299</v>
+      </c>
+      <c r="D138" t="s">
+        <v>301</v>
+      </c>
+      <c r="E138" t="s">
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>